<commit_message>
Sync updated STACK master workbook
</commit_message>
<xml_diff>
--- a/STACK_Policy_Master.xlsx
+++ b/STACK_Policy_Master.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaychittooran/Downloads/STACK_Policy_Automation_GitHub_Package/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaychittooran/Documents/STACK Policy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4633E724-7C17-8648-A6C0-3070EDB48F9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6895A3F-E226-3C4D-9359-15DFBFD4D186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1676,13 +1676,13 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>18</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="E6" s="2">
         <f>COUNTIFS('State Scores'!G2:G51,"&gt;=60",'State Scores'!G2:G51,"&lt;80")</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="E8" s="2">
         <f>COUNTIF('State Scores'!G2:G51,"&lt;40")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="B10" s="2">
         <f>AVERAGE('State Scores'!G2:G51)</f>
-        <v>59.11</v>
+        <v>58.06</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -2482,20 +2482,20 @@
         <v>310</v>
       </c>
       <c r="C2" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E2" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F2" s="7">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="G2" s="8">
         <f t="shared" ref="G2:G33" si="0">ROUND(20*(0.35*C2+0.15*D2+0.25*E2+0.25*F2),1)</f>
-        <v>72.5</v>
+        <v>20</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>54</v>

</xml_diff>